<commit_message>
Add fourth 1688 candidate to profit calculation
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EnTeSu63RHr4o5fRYRPgMW
</commit_message>
<xml_diff>
--- a/OEMリサーチ_スプレッドシート用.xlsx
+++ b/OEMリサーチ_スプレッドシート用.xlsx
@@ -1133,7 +1133,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="854" uniqueCount="476">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="856" uniqueCount="478">
   <si>
     <r>
       <rPr>
@@ -4208,6 +4208,86 @@
       <t xml:space="preserve">元</t>
     </r>
   </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Noto Sans JP"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">D </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">義烏嘉成・厚手ボア裏 高伸縮 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Noto Sans JP"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">6.99</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">元（工場）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Noto Sans JP"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">D </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">同上を</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Noto Sans JP"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1,980</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">円で販売</t>
+    </r>
+  </si>
 </sst>
 </file>
 
@@ -40741,93 +40821,121 @@
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="22"/>
-      <c r="B7" s="9"/>
-      <c r="C7" s="37"/>
-      <c r="D7" s="37"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="27" t="str">
+      <c r="A7" s="22" t="s">
+        <v>476</v>
+      </c>
+      <c r="B7" s="9" t="n">
+        <v>1780</v>
+      </c>
+      <c r="C7" s="37" t="n">
+        <v>6.99</v>
+      </c>
+      <c r="D7" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="9" t="n">
+        <v>120</v>
+      </c>
+      <c r="F7" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="G7" s="27" t="n">
         <f aca="false">IF(B7="","",(C7+D7)*設定!$B$6*(1+設定!$B$7)+E7+F7)</f>
-        <v/>
-      </c>
-      <c r="H7" s="27" t="str">
+        <v>356.1795</v>
+      </c>
+      <c r="H7" s="27" t="n">
         <f aca="false">IF(B7="","",ROUND(G7*設定!$B$8+G7*(1+設定!$B$8)*設定!$B$9,0))</f>
-        <v/>
-      </c>
-      <c r="I7" s="27" t="str">
+        <v>75</v>
+      </c>
+      <c r="I7" s="27" t="n">
         <f aca="false">IF(B7="","",ROUND(B7*設定!$B$10,0)+設定!$B$11+設定!$B$12)</f>
-        <v/>
-      </c>
-      <c r="J7" s="38" t="str">
+        <v>512</v>
+      </c>
+      <c r="J7" s="38" t="n">
         <f aca="false">IF(B7="","",B7-G7-H7-I7)</f>
-        <v/>
-      </c>
-      <c r="K7" s="39" t="str">
+        <v>836.8205</v>
+      </c>
+      <c r="K7" s="39" t="n">
         <f aca="false">IF(B7="","",IFERROR(J7/B7,""))</f>
-        <v/>
-      </c>
-      <c r="L7" s="39" t="str">
+        <v>0.470123876404494</v>
+      </c>
+      <c r="L7" s="39" t="n">
         <f aca="false">IF(B7="","",IFERROR(J7/(G7+H7),""))</f>
-        <v/>
-      </c>
-      <c r="M7" s="27" t="str">
+        <v>1.94077060713694</v>
+      </c>
+      <c r="M7" s="27" t="n">
         <f aca="false">IF(B7="","",IF(J7&lt;=0,"赤字",ROUNDUP(設定!$B$3/J7,0)))</f>
-        <v/>
-      </c>
-      <c r="N7" s="27" t="str">
+        <v>60</v>
+      </c>
+      <c r="N7" s="27" t="n">
         <f aca="false">IF(B7="","",IFERROR(ROUNDDOWN(設定!$B$4/(G7+H7),0),""))</f>
-        <v/>
-      </c>
-      <c r="O7" s="9"/>
+        <v>115</v>
+      </c>
+      <c r="O7" s="9" t="n">
+        <v>2</v>
+      </c>
       <c r="P7" s="28" t="str">
         <f aca="false">IF(B7="","",IF(J7&lt;=0,"× 赤字",IF(AND(K7&gt;=設定!$B$22,J7&gt;=設定!$B$23),IF(AND(O7&lt;&gt;"",N7&lt;O7),"△ 予算不足","○ OK"),"△ 利益薄い")))</f>
-        <v/>
+        <v>○ OK</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="22"/>
-      <c r="B8" s="9"/>
-      <c r="C8" s="37"/>
-      <c r="D8" s="37"/>
-      <c r="E8" s="9"/>
-      <c r="F8" s="9"/>
-      <c r="G8" s="27" t="str">
+      <c r="A8" s="22" t="s">
+        <v>477</v>
+      </c>
+      <c r="B8" s="9" t="n">
+        <v>1980</v>
+      </c>
+      <c r="C8" s="37" t="n">
+        <v>6.99</v>
+      </c>
+      <c r="D8" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="9" t="n">
+        <v>120</v>
+      </c>
+      <c r="F8" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="G8" s="27" t="n">
         <f aca="false">IF(B8="","",(C8+D8)*設定!$B$6*(1+設定!$B$7)+E8+F8)</f>
-        <v/>
-      </c>
-      <c r="H8" s="27" t="str">
+        <v>356.1795</v>
+      </c>
+      <c r="H8" s="27" t="n">
         <f aca="false">IF(B8="","",ROUND(G8*設定!$B$8+G8*(1+設定!$B$8)*設定!$B$9,0))</f>
-        <v/>
-      </c>
-      <c r="I8" s="27" t="str">
+        <v>75</v>
+      </c>
+      <c r="I8" s="27" t="n">
         <f aca="false">IF(B8="","",ROUND(B8*設定!$B$10,0)+設定!$B$11+設定!$B$12)</f>
-        <v/>
-      </c>
-      <c r="J8" s="38" t="str">
+        <v>528</v>
+      </c>
+      <c r="J8" s="38" t="n">
         <f aca="false">IF(B8="","",B8-G8-H8-I8)</f>
-        <v/>
-      </c>
-      <c r="K8" s="39" t="str">
+        <v>1020.8205</v>
+      </c>
+      <c r="K8" s="39" t="n">
         <f aca="false">IF(B8="","",IFERROR(J8/B8,""))</f>
-        <v/>
-      </c>
-      <c r="L8" s="39" t="str">
+        <v>0.515565909090909</v>
+      </c>
+      <c r="L8" s="39" t="n">
         <f aca="false">IF(B8="","",IFERROR(J8/(G8+H8),""))</f>
-        <v/>
-      </c>
-      <c r="M8" s="27" t="str">
+        <v>2.36750703593283</v>
+      </c>
+      <c r="M8" s="27" t="n">
         <f aca="false">IF(B8="","",IF(J8&lt;=0,"赤字",ROUNDUP(設定!$B$3/J8,0)))</f>
-        <v/>
-      </c>
-      <c r="N8" s="27" t="str">
+        <v>49</v>
+      </c>
+      <c r="N8" s="27" t="n">
         <f aca="false">IF(B8="","",IFERROR(ROUNDDOWN(設定!$B$4/(G8+H8),0),""))</f>
-        <v/>
-      </c>
-      <c r="O8" s="9"/>
+        <v>115</v>
+      </c>
+      <c r="O8" s="9" t="n">
+        <v>2</v>
+      </c>
       <c r="P8" s="28" t="str">
         <f aca="false">IF(B8="","",IF(J8&lt;=0,"× 赤字",IF(AND(K8&gt;=設定!$B$22,J8&gt;=設定!$B$23),IF(AND(O8&lt;&gt;"",N8&lt;O8),"△ 予算不足","○ OK"),"△ 利益薄い")))</f>
-        <v/>
+        <v>○ OK</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Add purchasing agent comparison sheet with cost simulation
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EnTeSu63RHr4o5fRYRPgMW
</commit_message>
<xml_diff>
--- a/OEMリサーチ_スプレッドシート用.xlsx
+++ b/OEMリサーチ_スプレッドシート用.xlsx
@@ -16,6 +16,7 @@
     <sheet name="上位10件データ" sheetId="6" state="visible" r:id="rId8"/>
     <sheet name="ライバル調査" sheetId="7" state="visible" r:id="rId9"/>
     <sheet name="利益計算" sheetId="8" state="visible" r:id="rId10"/>
+    <sheet name="代行業者比較" sheetId="9" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">セラーリスト!$A$1:$O$201</definedName>
@@ -1133,7 +1134,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="856" uniqueCount="478">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="931" uniqueCount="547">
   <si>
     <r>
       <rPr>
@@ -4288,6 +4289,1219 @@
       <t xml:space="preserve">円で販売</t>
     </r>
   </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="13"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">仕入れ代行業者 比較（</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="13"/>
+        <rFont val="Noto Sans JP"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2026</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="13"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">年</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="13"/>
+        <rFont val="Noto Sans JP"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="13"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">月時点の公開情報。契約前に各社公式で要確認）</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">ラクマート（一般会員）</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Noto Sans JP"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">THE CKB</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（フリープラン）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">イーウーパスポート（</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Noto Sans JP"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">FREE</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">会員）</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">■ 基本情報</t>
+  </si>
+  <si>
+    <t xml:space="preserve">月額料金</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans JP"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">円</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans JP"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">円（スタンダード </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans JP"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">9,800</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">円）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans JP"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">円（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans JP"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">GOLD 29,800</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">円）</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">有料プランは仕入れが月数十万円以上になってから検討</t>
+  </si>
+  <si>
+    <t xml:space="preserve">仕入れ代行手数料</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">商品代の</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans JP"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5%</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（累計利用額で最低</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans JP"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3%</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">まで下がる）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans JP"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0%</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans JP"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">B2B</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">仕入れ）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans JP"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5%</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans JP"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">GOLD</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">以上は</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans JP"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0%</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">）</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">無料プランの目安・制限</t>
+  </si>
+  <si>
+    <t xml:space="preserve">制限なし</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">推奨は月</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans JP"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">万円までの仕入れ。入出庫料はスタンダード以上で無料</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans JP"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">GOLD</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">は専任担当付き</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">フリープランで追加になる費用は要問い合わせ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">検品</t>
+  </si>
+  <si>
+    <t xml:space="preserve">基本検品は手数料に含む（詳細検品は有料）</t>
+  </si>
+  <si>
+    <t xml:space="preserve">オプション（有料）</t>
+  </si>
+  <si>
+    <t xml:space="preserve">オプション（要確認）</t>
+  </si>
+  <si>
+    <t xml:space="preserve">今回は糸くず・汚れの確認が重要。詳細検品の料金を聞く</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans JP"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">FBA</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">倉庫への直送</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">対応（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans JP"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Amazon</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">連携あり）</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">対応（要確認）</t>
+  </si>
+  <si>
+    <t xml:space="preserve">最初は自宅に届けて自分で検品するのがおすすめ</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans JP"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">OEM</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（タグ・袋・ロゴ）</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">対応</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans JP"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">OEM</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">資材はスタンダード以上</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">ブランドタグの作成費・最小数を聞く</t>
+  </si>
+  <si>
+    <t xml:space="preserve">向いている人</t>
+  </si>
+  <si>
+    <t xml:space="preserve">少量から始めたい初心者</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">仕入れが月</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans JP"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">万円以内の少量テスト</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">仕入れ量が多い中・上級者</t>
+  </si>
+  <si>
+    <t xml:space="preserve">■ 初回注文のコスト試算（黄色に見積もりを入力）</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ラクマート</t>
+  </si>
+  <si>
+    <t xml:space="preserve">THE CKB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">イーウーパスポート</t>
+  </si>
+  <si>
+    <t xml:space="preserve">商品代金（元）</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">例：候補</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans JP"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">D</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">を</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans JP"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">115</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">個（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans JP"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">万円予算の上限）。注文内容に合わせて変更</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">為替（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans JP"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">元＝円）</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">設定シートと連動</t>
+  </si>
+  <si>
+    <t xml:space="preserve">商品代金（円）</t>
+  </si>
+  <si>
+    <t xml:space="preserve">代行手数料率</t>
+  </si>
+  <si>
+    <t xml:space="preserve">公開情報より</t>
+  </si>
+  <si>
+    <t xml:space="preserve">代行手数料（円）</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">総重量（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans JP"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">kg</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans JP"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">個</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans JP"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">100g×115</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">個の仮定。業者の実測で更新</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">国際送料（円</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans JP"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/kg</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">航空便の相場は</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans JP"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1kg</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">あたり約</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans JP"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">400</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">〜</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans JP"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">600</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">円（まとめて送る場合）。見積もりで更新</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">国際送料（円）</t>
+  </si>
+  <si>
+    <t xml:space="preserve">検品・入出庫料（円）</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">見積もり待ち（仮に</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans JP"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">円）</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">タグ付け・袋入れ（円）</t>
+  </si>
+  <si>
+    <t xml:space="preserve">月額料金（円）</t>
+  </si>
+  <si>
+    <t xml:space="preserve">無料プランの場合</t>
+  </si>
+  <si>
+    <t xml:space="preserve">合計（関税・消費税は除く）</t>
+  </si>
+  <si>
+    <t xml:space="preserve">個数</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans JP"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">個あたり（円）</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">利益計算シートの『仕入れ原価』と比べる</t>
+  </si>
+  <si>
+    <t xml:space="preserve">■ 業者に問い合わせて確認すること（見積もり依頼で一緒に聞く）</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans JP"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1. 1688</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">の商品</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans JP"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">URL</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">と数量を渡して、商品代・手数料・国際送料（航空便）の合計見積もり</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans JP"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">詳細検品（糸くず・汚れ・縫製）の料金と、不良品があったときの返品・交換の対応</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans JP"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">ブランドタグ（織りネーム／下げ札）の作成費・最小ロット、袋の入れ替え費用</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans JP"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4. FBA</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">倉庫への直送の費用と、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans JP"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">FBA</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">ラベル（商品ラベル）の貼り付け費用</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans JP"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">サンプル（数個）だけを先に送ってもらうときの送料</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">出典</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF595959"/>
+        <rFont val="Noto Sans JP"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">: THE CKB</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">料金ページ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF595959"/>
+        <rFont val="Noto Sans JP"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">https://www.theckb.com/price/ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／ イーウーパスポート </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF595959"/>
+        <rFont val="Noto Sans JP"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">https://yiwupassport.com/membership-details/ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／ ラクマート </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF595959"/>
+        <rFont val="Noto Sans JP"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">https://www.rakumart.com/tollVipApplyFor </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">ほか比較記事（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF595959"/>
+        <rFont val="Noto Sans JP"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2026</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">年）</t>
+    </r>
+  </si>
 </sst>
 </file>
 
@@ -4304,7 +5518,7 @@
     <numFmt numFmtId="171" formatCode="#,##0.0"/>
     <numFmt numFmtId="172" formatCode="#,##0;\-#,##0"/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="28">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -4451,6 +5665,40 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b val="true"/>
+      <sz val="13"/>
+      <name val="WenQuanYi Zen Hei"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="13"/>
+      <name val="Noto Sans JP"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="WenQuanYi Zen Hei"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="WenQuanYi Zen Hei"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Noto Sans JP"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -4533,7 +5781,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="58">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -4691,6 +5939,78 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="167" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="25" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="26" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="25" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="27" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="27" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -49644,4 +50964,475 @@
   </headerFooter>
   <legacyDrawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:E35"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="46"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="40" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="29.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="41" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" s="41" t="s">
+        <v>479</v>
+      </c>
+      <c r="C3" s="42" t="s">
+        <v>480</v>
+      </c>
+      <c r="D3" s="41" t="s">
+        <v>481</v>
+      </c>
+      <c r="E3" s="41" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="43" t="s">
+        <v>482</v>
+      </c>
+      <c r="B4" s="43"/>
+      <c r="C4" s="43"/>
+      <c r="D4" s="43"/>
+      <c r="E4" s="43"/>
+    </row>
+    <row r="5" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="44" t="s">
+        <v>483</v>
+      </c>
+      <c r="B5" s="45" t="s">
+        <v>484</v>
+      </c>
+      <c r="C5" s="45" t="s">
+        <v>485</v>
+      </c>
+      <c r="D5" s="45" t="s">
+        <v>486</v>
+      </c>
+      <c r="E5" s="44" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="44" t="s">
+        <v>488</v>
+      </c>
+      <c r="B6" s="44" t="s">
+        <v>489</v>
+      </c>
+      <c r="C6" s="45" t="s">
+        <v>490</v>
+      </c>
+      <c r="D6" s="45" t="s">
+        <v>491</v>
+      </c>
+      <c r="E6" s="45"/>
+    </row>
+    <row r="7" customFormat="false" ht="42.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="44" t="s">
+        <v>492</v>
+      </c>
+      <c r="B7" s="44" t="s">
+        <v>493</v>
+      </c>
+      <c r="C7" s="44" t="s">
+        <v>494</v>
+      </c>
+      <c r="D7" s="45" t="s">
+        <v>495</v>
+      </c>
+      <c r="E7" s="44" t="s">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="44" t="s">
+        <v>497</v>
+      </c>
+      <c r="B8" s="44" t="s">
+        <v>498</v>
+      </c>
+      <c r="C8" s="44" t="s">
+        <v>499</v>
+      </c>
+      <c r="D8" s="44" t="s">
+        <v>500</v>
+      </c>
+      <c r="E8" s="44" t="s">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="29.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="45" t="s">
+        <v>502</v>
+      </c>
+      <c r="B9" s="44" t="s">
+        <v>503</v>
+      </c>
+      <c r="C9" s="44" t="s">
+        <v>504</v>
+      </c>
+      <c r="D9" s="44" t="s">
+        <v>504</v>
+      </c>
+      <c r="E9" s="44" t="s">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="29.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="45" t="s">
+        <v>506</v>
+      </c>
+      <c r="B10" s="44" t="s">
+        <v>507</v>
+      </c>
+      <c r="C10" s="45" t="s">
+        <v>508</v>
+      </c>
+      <c r="D10" s="44" t="s">
+        <v>507</v>
+      </c>
+      <c r="E10" s="44" t="s">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="29.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="44" t="s">
+        <v>510</v>
+      </c>
+      <c r="B11" s="44" t="s">
+        <v>511</v>
+      </c>
+      <c r="C11" s="44" t="s">
+        <v>512</v>
+      </c>
+      <c r="D11" s="44" t="s">
+        <v>513</v>
+      </c>
+      <c r="E11" s="45"/>
+    </row>
+    <row r="13" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="41" t="s">
+        <v>514</v>
+      </c>
+      <c r="B13" s="41" t="s">
+        <v>515</v>
+      </c>
+      <c r="C13" s="42" t="s">
+        <v>516</v>
+      </c>
+      <c r="D13" s="41" t="s">
+        <v>517</v>
+      </c>
+      <c r="E13" s="41" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="29.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="44" t="s">
+        <v>518</v>
+      </c>
+      <c r="B14" s="46" t="n">
+        <f aca="false">6.99*115</f>
+        <v>803.85</v>
+      </c>
+      <c r="C14" s="46" t="n">
+        <f aca="false">6.99*115</f>
+        <v>803.85</v>
+      </c>
+      <c r="D14" s="46" t="n">
+        <f aca="false">6.99*115</f>
+        <v>803.85</v>
+      </c>
+      <c r="E14" s="44" t="s">
+        <v>519</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="44" t="s">
+        <v>520</v>
+      </c>
+      <c r="B15" s="47" t="n">
+        <f aca="false">設定!$B$6</f>
+        <v>21</v>
+      </c>
+      <c r="C15" s="47" t="n">
+        <f aca="false">設定!$B$6</f>
+        <v>21</v>
+      </c>
+      <c r="D15" s="47" t="n">
+        <f aca="false">設定!$B$6</f>
+        <v>21</v>
+      </c>
+      <c r="E15" s="44" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="44" t="s">
+        <v>522</v>
+      </c>
+      <c r="B16" s="48" t="n">
+        <f aca="false">B14*B15</f>
+        <v>16880.85</v>
+      </c>
+      <c r="C16" s="48" t="n">
+        <f aca="false">C14*C15</f>
+        <v>16880.85</v>
+      </c>
+      <c r="D16" s="48" t="n">
+        <f aca="false">D14*D15</f>
+        <v>16880.85</v>
+      </c>
+      <c r="E16" s="45"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="44" t="s">
+        <v>523</v>
+      </c>
+      <c r="B17" s="49" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C17" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="49" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E17" s="44" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="44" t="s">
+        <v>525</v>
+      </c>
+      <c r="B18" s="48" t="n">
+        <f aca="false">B16*B17</f>
+        <v>844.0425</v>
+      </c>
+      <c r="C18" s="48" t="n">
+        <f aca="false">C16*C17</f>
+        <v>0</v>
+      </c>
+      <c r="D18" s="48" t="n">
+        <f aca="false">D16*D17</f>
+        <v>844.0425</v>
+      </c>
+      <c r="E18" s="45"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="44" t="s">
+        <v>526</v>
+      </c>
+      <c r="B19" s="50" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="C19" s="50" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="D19" s="50" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="E19" s="45" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="29.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="44" t="s">
+        <v>528</v>
+      </c>
+      <c r="B20" s="51" t="n">
+        <v>600</v>
+      </c>
+      <c r="C20" s="51" t="n">
+        <v>600</v>
+      </c>
+      <c r="D20" s="51" t="n">
+        <v>600</v>
+      </c>
+      <c r="E20" s="44" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="44" t="s">
+        <v>530</v>
+      </c>
+      <c r="B21" s="48" t="n">
+        <f aca="false">B19*B20</f>
+        <v>6900</v>
+      </c>
+      <c r="C21" s="48" t="n">
+        <f aca="false">C19*C20</f>
+        <v>6900</v>
+      </c>
+      <c r="D21" s="48" t="n">
+        <f aca="false">D19*D20</f>
+        <v>6900</v>
+      </c>
+      <c r="E21" s="45"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="44" t="s">
+        <v>531</v>
+      </c>
+      <c r="B22" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" s="44" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="44" t="s">
+        <v>533</v>
+      </c>
+      <c r="B23" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" s="44" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="44" t="s">
+        <v>534</v>
+      </c>
+      <c r="B24" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" s="44" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="52" t="s">
+        <v>536</v>
+      </c>
+      <c r="B25" s="53" t="n">
+        <f aca="false">B16+B18+B21+B22+B23+B24</f>
+        <v>24624.8925</v>
+      </c>
+      <c r="C25" s="53" t="n">
+        <f aca="false">C16+C18+C21+C22+C23+C24</f>
+        <v>23780.85</v>
+      </c>
+      <c r="D25" s="53" t="n">
+        <f aca="false">D16+D18+D21+D22+D23+D24</f>
+        <v>24624.8925</v>
+      </c>
+      <c r="E25" s="52"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="44" t="s">
+        <v>537</v>
+      </c>
+      <c r="B26" s="51" t="n">
+        <v>115</v>
+      </c>
+      <c r="C26" s="51" t="n">
+        <v>115</v>
+      </c>
+      <c r="D26" s="51" t="n">
+        <v>115</v>
+      </c>
+      <c r="E26" s="45"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="54" t="s">
+        <v>538</v>
+      </c>
+      <c r="B27" s="53" t="n">
+        <f aca="false">IFERROR(B25/B26,"")</f>
+        <v>214.1295</v>
+      </c>
+      <c r="C27" s="53" t="n">
+        <f aca="false">IFERROR(C25/C26,"")</f>
+        <v>206.79</v>
+      </c>
+      <c r="D27" s="53" t="n">
+        <f aca="false">IFERROR(D25/D26,"")</f>
+        <v>214.1295</v>
+      </c>
+      <c r="E27" s="52" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="55" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="56" t="s">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="56" t="s">
+        <v>542</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="56" t="s">
+        <v>543</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="56" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="56" t="s">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="57" t="s">
+        <v>546</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>